<commit_message>
fix: DOCX import — fix missing Q23, x^{2+} display bug, image-variant recovery
- Frontend: convertV1 now uses server detectedType — chemistry converter
  only for chemistry content, prevents x^2+x → x^{2+}x in math
- Backend: preCleanText regex tightened — bare numbers like "7 A" no longer
  become false question markers (requires word start after uppercase)
- Backend: filterSequentialMarkers — added debug logging for dropped markers
- Backend: extractQuestion — image-variant recovery for questions with <2
  text variants but image markers present
- Backend: validateWithAI — now includes 0-variant questions for AI repair

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sinflar/9 A Iqtisod - Dekabr blok test.xlsx
+++ b/sinflar/9 A Iqtisod - Dekabr blok test.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="6975"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>№</t>
   </si>
@@ -161,12 +161,6 @@
   </si>
   <si>
     <t>Yoqubjonova Dilnura</t>
-  </si>
-  <si>
-    <t>Zamonov Shohruh</t>
-  </si>
-  <si>
-    <t>Rahimov Adham</t>
   </si>
 </sst>
 </file>
@@ -898,55 +892,55 @@
     </xf>
   </cellXfs>
   <cellStyles count="49">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
-    <cellStyle name="Запятая" xfId="1" builtinId="3"/>
-    <cellStyle name="Денежный" xfId="2" builtinId="4"/>
-    <cellStyle name="Процент" xfId="3" builtinId="5"/>
-    <cellStyle name="Запятая [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Денежный [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Гиперссылка" xfId="6" builtinId="8"/>
-    <cellStyle name="Открывавшаяся гиперссылка" xfId="7" builtinId="9"/>
-    <cellStyle name="Примечание" xfId="8" builtinId="10"/>
-    <cellStyle name="Предупреждающий текст" xfId="9" builtinId="11"/>
-    <cellStyle name="Заголовок" xfId="10" builtinId="15"/>
-    <cellStyle name="Пояснительный текст" xfId="11" builtinId="53"/>
-    <cellStyle name="Заголовок 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Заголовок 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Заголовок 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Заголовок 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Ввод" xfId="16" builtinId="20"/>
-    <cellStyle name="Вывод" xfId="17" builtinId="21"/>
-    <cellStyle name="Вычисление" xfId="18" builtinId="22"/>
-    <cellStyle name="Проверить ячейку" xfId="19" builtinId="23"/>
-    <cellStyle name="Связанная ячейка" xfId="20" builtinId="24"/>
-    <cellStyle name="Итого" xfId="21" builtinId="25"/>
-    <cellStyle name="Хороший" xfId="22" builtinId="26"/>
-    <cellStyle name="Плохой" xfId="23" builtinId="27"/>
-    <cellStyle name="Нейтральный" xfId="24" builtinId="28"/>
-    <cellStyle name="Акцент1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% — Акцент1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% — Акцент1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% — Акцент1" xfId="28" builtinId="32"/>
-    <cellStyle name="Акцент2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% — Акцент2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% — Акцент2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% — Акцент2" xfId="32" builtinId="36"/>
-    <cellStyle name="Акцент3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% — Акцент3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% — Акцент3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% — Акцент3" xfId="36" builtinId="40"/>
-    <cellStyle name="Акцент4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% — Акцент4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% — Акцент4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% — Акцент4" xfId="40" builtinId="44"/>
-    <cellStyle name="Акцент5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% — Акцент5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% — Акцент5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% — Акцент5" xfId="44" builtinId="48"/>
-    <cellStyle name="Акцент6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% — Акцент6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% — Акцент6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% — Акцент6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <extLst>
@@ -1245,17 +1239,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G40"/>
-  <sheetFormatPr defaultColWidth="9.13333333333333" defaultRowHeight="26.25" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.12962962962963" defaultRowHeight="25.8" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="6" style="2" customWidth="1"/>
-    <col min="2" max="2" width="43.8857142857143" style="2" customWidth="1"/>
-    <col min="3" max="3" width="22.8857142857143" style="2" customWidth="1"/>
-    <col min="4" max="4" width="17.3809523809524" style="3" customWidth="1"/>
-    <col min="5" max="5" width="11.447619047619" style="2" customWidth="1"/>
+    <col min="2" max="2" width="43.8888888888889" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.8888888888889" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17.3796296296296" style="3" customWidth="1"/>
+    <col min="5" max="5" width="11.4444444444444" style="2" customWidth="1"/>
     <col min="6" max="6" width="11.6666666666667" style="2" customWidth="1"/>
-    <col min="7" max="7" width="22.8857142857143" style="2" customWidth="1"/>
-    <col min="8" max="8" width="8.22857142857143" style="2" customWidth="1"/>
-    <col min="9" max="16384" width="9.13333333333333" style="4"/>
+    <col min="7" max="7" width="22.8888888888889" style="2" customWidth="1"/>
+    <col min="8" max="8" width="8.23148148148148" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="9.12962962962963" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1798,11 +1792,11 @@
         <v>13</v>
       </c>
       <c r="F22" s="13">
-        <f>C22*3.1+D22*2.1+E22*1.1</f>
+        <f t="shared" si="0"/>
         <v>124.5</v>
       </c>
       <c r="G22" s="15">
-        <f>F22/189</f>
+        <f t="shared" si="1"/>
         <v>0.658730158730159</v>
       </c>
     </row>
@@ -1823,11 +1817,11 @@
         <v>10</v>
       </c>
       <c r="F23" s="13">
-        <f>C23*3.1+D23*2.1+E23*1.1</f>
+        <f t="shared" si="0"/>
         <v>124.4</v>
       </c>
       <c r="G23" s="15">
-        <f>F23/189</f>
+        <f t="shared" si="1"/>
         <v>0.658201058201058</v>
       </c>
     </row>
@@ -1848,11 +1842,11 @@
         <v>10</v>
       </c>
       <c r="F24" s="13">
-        <f>C24*3.1+D24*2.1+E24*1.1</f>
+        <f t="shared" si="0"/>
         <v>123.3</v>
       </c>
       <c r="G24" s="15">
-        <f>F24/189</f>
+        <f t="shared" si="1"/>
         <v>0.652380952380952</v>
       </c>
     </row>
@@ -1873,11 +1867,11 @@
         <v>14</v>
       </c>
       <c r="F25" s="13">
-        <f>C25*3.1+D25*2.1+E25*1.1</f>
+        <f t="shared" si="0"/>
         <v>122.4</v>
       </c>
       <c r="G25" s="15">
-        <f>F25/189</f>
+        <f t="shared" si="1"/>
         <v>0.647619047619048</v>
       </c>
     </row>
@@ -1898,11 +1892,11 @@
         <v>9</v>
       </c>
       <c r="F26" s="13">
-        <f>C26*3.1+D26*2.1+E26*1.1</f>
+        <f t="shared" si="0"/>
         <v>122</v>
       </c>
       <c r="G26" s="15">
-        <f>F26/189</f>
+        <f t="shared" si="1"/>
         <v>0.645502645502646</v>
       </c>
     </row>
@@ -1923,11 +1917,11 @@
         <v>11</v>
       </c>
       <c r="F27" s="13">
-        <f>C27*3.1+D27*2.1+E27*1.1</f>
+        <f t="shared" si="0"/>
         <v>120.4</v>
       </c>
       <c r="G27" s="15">
-        <f>F27/189</f>
+        <f t="shared" si="1"/>
         <v>0.637037037037037</v>
       </c>
     </row>
@@ -1948,11 +1942,11 @@
         <v>14</v>
       </c>
       <c r="F28" s="13">
-        <f>C28*3.1+D28*2.1+E28*1.1</f>
+        <f t="shared" si="0"/>
         <v>119.5</v>
       </c>
       <c r="G28" s="15">
-        <f>F28/189</f>
+        <f t="shared" si="1"/>
         <v>0.632275132275132</v>
       </c>
     </row>
@@ -1973,11 +1967,11 @@
         <v>4</v>
       </c>
       <c r="F29" s="13">
-        <f>C29*3.1+D29*2.1+E29*1.1</f>
+        <f t="shared" si="0"/>
         <v>118.7</v>
       </c>
       <c r="G29" s="15">
-        <f>F29/189</f>
+        <f t="shared" si="1"/>
         <v>0.628042328042328</v>
       </c>
     </row>
@@ -1998,11 +1992,11 @@
         <v>9</v>
       </c>
       <c r="F30" s="13">
-        <f>C30*3.1+D30*2.1+E30*1.1</f>
+        <f t="shared" si="0"/>
         <v>116.9</v>
       </c>
       <c r="G30" s="15">
-        <f>F30/189</f>
+        <f t="shared" si="1"/>
         <v>0.618518518518519</v>
       </c>
     </row>
@@ -2023,11 +2017,11 @@
         <v>14</v>
       </c>
       <c r="F31" s="13">
-        <f>C31*3.1+D31*2.1+E31*1.1</f>
+        <f t="shared" si="0"/>
         <v>116.3</v>
       </c>
       <c r="G31" s="15">
-        <f>F31/189</f>
+        <f t="shared" si="1"/>
         <v>0.615343915343915</v>
       </c>
     </row>
@@ -2048,11 +2042,11 @@
         <v>14</v>
       </c>
       <c r="F32" s="13">
-        <f>C32*3.1+D32*2.1+E32*1.1</f>
+        <f t="shared" si="0"/>
         <v>112.1</v>
       </c>
       <c r="G32" s="15">
-        <f>F32/189</f>
+        <f t="shared" si="1"/>
         <v>0.593121693121693</v>
       </c>
     </row>
@@ -2073,11 +2067,11 @@
         <v>11</v>
       </c>
       <c r="F33" s="13">
-        <f>C33*3.1+D33*2.1+E33*1.1</f>
+        <f t="shared" si="0"/>
         <v>112</v>
       </c>
       <c r="G33" s="15">
-        <f>F33/189</f>
+        <f t="shared" si="1"/>
         <v>0.592592592592593</v>
       </c>
     </row>
@@ -2098,11 +2092,11 @@
         <v>12</v>
       </c>
       <c r="F34" s="13">
-        <f>C34*3.1+D34*2.1+E34*1.1</f>
+        <f t="shared" si="0"/>
         <v>110.1</v>
       </c>
       <c r="G34" s="15">
-        <f>F34/189</f>
+        <f t="shared" si="1"/>
         <v>0.582539682539683</v>
       </c>
     </row>
@@ -2123,11 +2117,11 @@
         <v>9</v>
       </c>
       <c r="F35" s="13">
-        <f>C35*3.1+D35*2.1+E35*1.1</f>
+        <f t="shared" si="0"/>
         <v>107.6</v>
       </c>
       <c r="G35" s="15">
-        <f>F35/189</f>
+        <f t="shared" si="1"/>
         <v>0.569312169312169</v>
       </c>
     </row>
@@ -2148,11 +2142,11 @@
         <v>7</v>
       </c>
       <c r="F36" s="16">
-        <f>C36*3.1+D36*2.1+E36*1.1</f>
+        <f t="shared" si="0"/>
         <v>101.4</v>
       </c>
       <c r="G36" s="18">
-        <f>F36/189</f>
+        <f t="shared" si="1"/>
         <v>0.536507936507936</v>
       </c>
     </row>
@@ -2173,11 +2167,11 @@
         <v>9</v>
       </c>
       <c r="F37" s="16">
-        <f>C37*3.1+D37*2.1+E37*1.1</f>
+        <f t="shared" si="0"/>
         <v>99.5</v>
       </c>
       <c r="G37" s="18">
-        <f>F37/189</f>
+        <f t="shared" si="1"/>
         <v>0.526455026455027</v>
       </c>
     </row>
@@ -2198,11 +2192,11 @@
         <v>12</v>
       </c>
       <c r="F38" s="16">
-        <f>C38*3.1+D38*2.1+E38*1.1</f>
+        <f t="shared" si="0"/>
         <v>96.5</v>
       </c>
       <c r="G38" s="18">
-        <f>F38/189</f>
+        <f t="shared" si="1"/>
         <v>0.510582010582011</v>
       </c>
     </row>
@@ -2210,50 +2204,16 @@
       <c r="A39" s="16">
         <v>39</v>
       </c>
-      <c r="B39" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="C39" s="16">
-        <v>18</v>
-      </c>
-      <c r="D39" s="17">
-        <v>14</v>
-      </c>
-      <c r="E39" s="16">
-        <v>8</v>
-      </c>
-      <c r="F39" s="16">
-        <f>C39*3.1+D39*2.1+E39*1.1</f>
-        <v>94</v>
-      </c>
-      <c r="G39" s="18">
-        <f>F39/189</f>
-        <v>0.497354497354497</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
+      <c r="B39" s="16"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="16"/>
+      <c r="F39" s="16"/>
+      <c r="G39" s="18"/>
+    </row>
+    <row r="40" spans="1:1">
       <c r="A40" s="16">
         <v>40</v>
-      </c>
-      <c r="B40" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="C40" s="16">
-        <v>15</v>
-      </c>
-      <c r="D40" s="17">
-        <v>17</v>
-      </c>
-      <c r="E40" s="16">
-        <v>6</v>
-      </c>
-      <c r="F40" s="16">
-        <f>C40*3.1+D40*2.1+E40*1.1</f>
-        <v>88.8</v>
-      </c>
-      <c r="G40" s="18">
-        <f>F40/189</f>
-        <v>0.46984126984127</v>
       </c>
     </row>
   </sheetData>
@@ -2270,204 +2230,204 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:A40"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" ht="15.75" spans="1:1">
+    <row r="1" ht="15.6" spans="1:1">
       <c r="A1" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="15.75" spans="1:1">
+    <row r="2" ht="15.6" spans="1:1">
       <c r="A2" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="3" ht="15.75" spans="1:1">
+    <row r="3" ht="15.6" spans="1:1">
       <c r="A3" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="4" ht="15.75" spans="1:1">
+    <row r="4" ht="15.6" spans="1:1">
       <c r="A4" s="1">
         <v>4</v>
       </c>
     </row>
-    <row r="5" ht="15.75" spans="1:1">
+    <row r="5" ht="15.6" spans="1:1">
       <c r="A5" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="6" ht="15.75" spans="1:1">
+    <row r="6" ht="15.6" spans="1:1">
       <c r="A6" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="7" ht="15.75" spans="1:1">
+    <row r="7" ht="15.6" spans="1:1">
       <c r="A7" s="1">
         <v>7</v>
       </c>
     </row>
-    <row r="8" ht="15.75" spans="1:1">
+    <row r="8" ht="15.6" spans="1:1">
       <c r="A8" s="1">
         <v>8</v>
       </c>
     </row>
-    <row r="9" ht="15.75" spans="1:1">
+    <row r="9" ht="15.6" spans="1:1">
       <c r="A9" s="1">
         <v>9</v>
       </c>
     </row>
-    <row r="10" ht="15.75" spans="1:1">
+    <row r="10" ht="15.6" spans="1:1">
       <c r="A10" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="11" ht="15.75" spans="1:1">
+    <row r="11" ht="15.6" spans="1:1">
       <c r="A11" s="1">
         <v>11</v>
       </c>
     </row>
-    <row r="12" ht="15.75" spans="1:1">
+    <row r="12" ht="15.6" spans="1:1">
       <c r="A12" s="1">
         <v>12</v>
       </c>
     </row>
-    <row r="13" ht="15.75" spans="1:1">
+    <row r="13" ht="15.6" spans="1:1">
       <c r="A13" s="1">
         <v>13</v>
       </c>
     </row>
-    <row r="14" ht="15.75" spans="1:1">
+    <row r="14" ht="15.6" spans="1:1">
       <c r="A14" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="15" ht="15.75" spans="1:1">
+    <row r="15" ht="15.6" spans="1:1">
       <c r="A15" s="1">
         <v>15</v>
       </c>
     </row>
-    <row r="16" ht="15.75" spans="1:1">
+    <row r="16" ht="15.6" spans="1:1">
       <c r="A16" s="1">
         <v>16</v>
       </c>
     </row>
-    <row r="17" ht="15.75" spans="1:1">
+    <row r="17" ht="15.6" spans="1:1">
       <c r="A17" s="1">
         <v>17</v>
       </c>
     </row>
-    <row r="18" ht="15.75" spans="1:1">
+    <row r="18" ht="15.6" spans="1:1">
       <c r="A18" s="1">
         <v>18</v>
       </c>
     </row>
-    <row r="19" ht="15.75" spans="1:1">
+    <row r="19" ht="15.6" spans="1:1">
       <c r="A19" s="1">
         <v>19</v>
       </c>
     </row>
-    <row r="20" ht="15.75" spans="1:1">
+    <row r="20" ht="15.6" spans="1:1">
       <c r="A20" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="21" ht="15.75" spans="1:1">
+    <row r="21" ht="15.6" spans="1:1">
       <c r="A21" s="1">
         <v>21</v>
       </c>
     </row>
-    <row r="22" ht="15.75" spans="1:1">
+    <row r="22" ht="15.6" spans="1:1">
       <c r="A22" s="1">
         <v>22</v>
       </c>
     </row>
-    <row r="23" ht="15.75" spans="1:1">
+    <row r="23" ht="15.6" spans="1:1">
       <c r="A23" s="1">
         <v>23</v>
       </c>
     </row>
-    <row r="24" ht="15.75" spans="1:1">
+    <row r="24" ht="15.6" spans="1:1">
       <c r="A24" s="1">
         <v>24</v>
       </c>
     </row>
-    <row r="25" ht="15.75" spans="1:1">
+    <row r="25" ht="15.6" spans="1:1">
       <c r="A25" s="1">
         <v>25</v>
       </c>
     </row>
-    <row r="26" ht="15.75" spans="1:1">
+    <row r="26" ht="15.6" spans="1:1">
       <c r="A26" s="1">
         <v>26</v>
       </c>
     </row>
-    <row r="27" ht="15.75" spans="1:1">
+    <row r="27" ht="15.6" spans="1:1">
       <c r="A27" s="1">
         <v>27</v>
       </c>
     </row>
-    <row r="28" ht="15.75" spans="1:1">
+    <row r="28" ht="15.6" spans="1:1">
       <c r="A28" s="1">
         <v>28</v>
       </c>
     </row>
-    <row r="29" ht="15.75" spans="1:1">
+    <row r="29" ht="15.6" spans="1:1">
       <c r="A29" s="1">
         <v>29</v>
       </c>
     </row>
-    <row r="30" ht="15.75" spans="1:1">
+    <row r="30" ht="15.6" spans="1:1">
       <c r="A30" s="1">
         <v>30</v>
       </c>
     </row>
-    <row r="31" ht="15.75" spans="1:1">
+    <row r="31" ht="15.6" spans="1:1">
       <c r="A31" s="1">
         <v>31</v>
       </c>
     </row>
-    <row r="32" ht="15.75" spans="1:1">
+    <row r="32" ht="15.6" spans="1:1">
       <c r="A32" s="1">
         <v>32</v>
       </c>
     </row>
-    <row r="33" ht="15.75" spans="1:1">
+    <row r="33" ht="15.6" spans="1:1">
       <c r="A33" s="1">
         <v>33</v>
       </c>
     </row>
-    <row r="34" ht="15.75" spans="1:1">
+    <row r="34" ht="15.6" spans="1:1">
       <c r="A34" s="1">
         <v>34</v>
       </c>
     </row>
-    <row r="35" ht="15.75" spans="1:1">
+    <row r="35" ht="15.6" spans="1:1">
       <c r="A35" s="1">
         <v>35</v>
       </c>
     </row>
-    <row r="36" ht="15.75" spans="1:1">
+    <row r="36" ht="15.6" spans="1:1">
       <c r="A36" s="1">
         <v>36</v>
       </c>
     </row>
-    <row r="37" ht="15.75" spans="1:1">
+    <row r="37" ht="15.6" spans="1:1">
       <c r="A37" s="1">
         <v>37</v>
       </c>
     </row>
-    <row r="38" ht="15.75" spans="1:1">
+    <row r="38" ht="15.6" spans="1:1">
       <c r="A38" s="1">
         <v>38</v>
       </c>
     </row>
-    <row r="39" ht="15.75" spans="1:1">
+    <row r="39" ht="15.6" spans="1:1">
       <c r="A39" s="1">
         <v>39</v>
       </c>
     </row>
-    <row r="40" ht="15.75" spans="1:1">
+    <row r="40" ht="15.6" spans="1:1">
       <c r="A40" s="1">
         <v>40</v>
       </c>
@@ -2482,7 +2442,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>